<commit_message>
feat(srv): codify physical invariants for dual ocp, primary 2x16 riser, n+1 power, and rear boot exclusion (INV-118 to INV-122)
</commit_message>
<xml_diff>
--- a/outputs/SAN/FC/SN3600B_FC/Config2_SN3600B_FC_Switch_EVALUATED_BOQ_Evaluated BOQ_MultiRank_Solutions.xlsx
+++ b/outputs/SAN/FC/SN3600B_FC/Config2_SN3600B_FC_Switch_EVALUATED_BOQ_Evaluated BOQ_MultiRank_Solutions.xlsx
@@ -1113,7 +1113,7 @@
         <v>Overall Physical Build Status</v>
       </c>
       <c r="B7" s="2" t="str">
-        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="8">
@@ -1121,7 +1121,7 @@
         <v>Dual-Brain Verification Badge</v>
       </c>
       <c r="B8" s="2" t="str">
-        <v>CANDIDATE DOCUMENT REVIEW PASSED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>CANDIDATE DOCUMENT REVIEW PASSED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="9">
@@ -1137,7 +1137,7 @@
         <v>QuickSpecs Citations Verified</v>
       </c>
       <c r="B10" s="2" t="str">
-        <v>32 Authoritative Citations</v>
+        <v>29 Authoritative Citations</v>
       </c>
     </row>
     <row r="11">
@@ -1145,7 +1145,7 @@
         <v>Evaluation Timestamp</v>
       </c>
       <c r="B11" s="2" t="str">
-        <v>2026-09-22T13:06:25.590Z</v>
+        <v>2026-09-23T13:30:56.388Z</v>
       </c>
     </row>
     <row r="13">
@@ -1181,7 +1181,7 @@
         <v>SAN bundle reconciliation</v>
       </c>
       <c r="C15" s="9">
-        <v>62636</v>
+        <v>61929</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -1190,7 +1190,7 @@
         <v>100%</v>
       </c>
       <c r="F15" s="8" t="str">
-        <v>CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="17">
@@ -1319,7 +1319,7 @@
         <v>Ready for Automated Cross-Verification</v>
       </c>
       <c r="G26" s="13" t="str">
-        <v>["[2, 3] HPE SN3600B 32Gb 24/8 switch (R7R97A) provides a 1U chassis with 24 physical SFP+ ports, 8 active ports enabled, and 8x 32Gb Short Wave SFP28 transceivers included in the base bundle.","[5, 6] HPE SN3600B 8-port upgrade license with transceiver kit (R7M09A) adds 8 licensed ports and 8x 32Gb SW SFP28 optics. Two kits expand licensed capacity to 24 ports and total optics to 24.","[7, 8] HPE Premier Flex LC/LC Multi-mode OM4 15m Cable (QK735A) uses LC connectors compatible with 32Gb SFP28 optics and supports 32Gb FC distances up to 100 meters.","[10, 11, 13] SN3600B architecture features an integrated single fixed AC power supply with 4 cooling fans and back-to-front airflow.","[1, 14, 15] HPE 3 Year Tech Care Basic wCDMR (HX2M2E) and HPE Installation Storage Switches Service (U5988E) are verified product-qualified services for switch model R7R97A."]</v>
+        <v>["HPE SN3600B 32Gb 24/8 FC Switch (R7R97A) provides 8 active ports out of 24 physical ports in a 1U form factor [1-3, 5] and includes 8x 32Gb Short Wave SFP28 transceivers [3].","HPE SN3600B 32Gb 8-port Upgrade License with Transceiver Kit (R7M09A) adds 8 active ports and 8x 32Gb SW SFP28 transceivers per kit [7, 8]. Qty 2 enables 16 additional ports (24 active ports total) and provides 16 transceivers [1, 5, 7, 8].","The base switch (8 transceivers) plus 2x R7M09A POD upgrade kits (16 transceivers) supply 24x 32Gb SW SFP28 transceivers in total [3, 7, 8], populating all 24 active ports and rendering standalone transceiver kit R6W26A redundant.","HPE Premier Flex LC/LC OM4 15m Cables (QK735A, qty 8) are fully supported multi-mode OM4 fiber optic cables for 32Gb FC transceivers [9, 10].","The SN3600B chassis includes an integrated single power supply with 4 built-in cooling fans and back-to-front airflow [11-13].","HPE Installation Service (HA113A1 / HA113A1#5GA) [14, 16] and HPE 3Y Tech Care Basic with DMR Service (HU4B3A3 / HU4B3A3#ZTL) [14, 15] are product-qualified services for switch model R7R97A."]</v>
       </c>
       <c r="H26" s="13" t="str">
         <v>✅ SYNCED (catalog_deltas &amp; master_registry)</v>
@@ -1334,7 +1334,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1357,7 +1357,7 @@
     </row>
     <row r="2">
       <c r="A2" s="15" t="str">
-        <v>Estimated CapEx: $62,636 | Alignment: 100% | Server Nodes: 1</v>
+        <v>Estimated CapEx: $61,929 | Alignment: 100% | Server Nodes: 1</v>
       </c>
     </row>
     <row r="3">
@@ -1435,7 +1435,7 @@
         <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
       </c>
       <c r="L4" s="13" t="str">
-        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="5">
@@ -1475,7 +1475,7 @@
         <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
       </c>
       <c r="L5" s="20" t="str">
-        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="6">
@@ -1515,12 +1515,12 @@
         <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
       </c>
       <c r="L6" s="13" t="str">
-        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="str">
-        <v>HX2M2E</v>
+        <v>HA113A1</v>
       </c>
       <c r="B7" s="19">
         <v>1</v>
@@ -1533,17 +1533,17 @@
         <v>1</v>
       </c>
       <c r="E7" s="20" t="str">
-        <v>HPE 3 Year Tech Care Basic wCDMR SN3600B 24/8 8p 32Gb SW SFP Switch Service</v>
+        <v>HPE Installation Service</v>
       </c>
       <c r="F7" s="20" t="str">
         <v>Standard Option</v>
       </c>
       <c r="G7" s="21">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="H7" s="21">
         <f>D7*G7</f>
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="I7" s="20" t="str">
         <v>Customer specified baseline component</v>
@@ -1555,12 +1555,12 @@
         <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
       </c>
       <c r="L7" s="20" t="str">
-        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="str">
-        <v>U5988E</v>
+        <v>HA113A1 5GA</v>
       </c>
       <c r="B8" s="16">
         <v>1</v>
@@ -1573,17 +1573,17 @@
         <v>1</v>
       </c>
       <c r="E8" s="13" t="str">
-        <v>HPE Installation Storage Switches Service</v>
+        <v>HPE LowEnd SAN/Edge Switch/HAFM Inst SVC</v>
       </c>
       <c r="F8" s="13" t="str">
         <v>Standard Option</v>
       </c>
       <c r="G8" s="17">
-        <v>480</v>
+        <v>537</v>
       </c>
       <c r="H8" s="17">
         <f>D8*G8</f>
-        <v>480</v>
+        <v>537</v>
       </c>
       <c r="I8" s="13" t="str">
         <v>Customer specified baseline component</v>
@@ -1595,51 +1595,131 @@
         <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
       </c>
       <c r="L8" s="13" t="str">
-        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="str">
+      <c r="A9" s="18" t="str">
+        <v>HU4B3A3</v>
+      </c>
+      <c r="B9" s="19">
+        <v>1</v>
+      </c>
+      <c r="C9" s="19">
+        <v>1</v>
+      </c>
+      <c r="D9" s="19">
+        <f>B9*C9</f>
+        <v>1</v>
+      </c>
+      <c r="E9" s="20" t="str">
+        <v>HPE 3Y Tech Care Basic with Defective Media Retention Service</v>
+      </c>
+      <c r="F9" s="20" t="str">
+        <v>Standard Option</v>
+      </c>
+      <c r="G9" s="21">
+        <v>0</v>
+      </c>
+      <c r="H9" s="21">
+        <f>D9*G9</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="20" t="str">
+        <v>Customer specified baseline component</v>
+      </c>
+      <c r="J9" s="20" t="str">
+        <v>CANDIDATE DOCUMENT REVIEW: PASS</v>
+      </c>
+      <c r="K9" s="20" t="str">
+        <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
+      </c>
+      <c r="L9" s="20" t="str">
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="str">
+        <v>HU4B3A3 ZTL</v>
+      </c>
+      <c r="B10" s="16">
+        <v>1</v>
+      </c>
+      <c r="C10" s="16">
+        <v>1</v>
+      </c>
+      <c r="D10" s="16">
+        <f>B10*C10</f>
+        <v>1</v>
+      </c>
+      <c r="E10" s="13" t="str">
+        <v>HPE SN3600B 24/8 8p 32G Swch Support</v>
+      </c>
+      <c r="F10" s="13" t="str">
+        <v>Standard Option</v>
+      </c>
+      <c r="G10" s="17">
+        <v>186</v>
+      </c>
+      <c r="H10" s="17">
+        <f>D10*G10</f>
+        <v>186</v>
+      </c>
+      <c r="I10" s="13" t="str">
+        <v>Customer specified baseline component</v>
+      </c>
+      <c r="J10" s="13" t="str">
+        <v>CANDIDATE DOCUMENT REVIEW: PASS</v>
+      </c>
+      <c r="K10" s="13" t="str">
+        <v>Remove standalone optics only where allocated to ports already supplied by base/upgrade bundles. Retain documented spares and remote-endpoint optics. Preserve the requested 24-port expansion.</v>
+      </c>
+      <c r="L10" s="13" t="str">
+        <v>LOCAL_RULE_CHECKED; CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="str">
         <v>SUBTOTAL / ESTIMATED CAPEX</v>
       </c>
-      <c r="B9" s="23" t="str">
+      <c r="B11" s="23" t="str">
         <v/>
       </c>
-      <c r="C9" s="23" t="str">
+      <c r="C11" s="23" t="str">
         <v/>
       </c>
-      <c r="D9" s="23" t="str">
+      <c r="D11" s="23" t="str">
         <v/>
       </c>
-      <c r="E9" s="23" t="str">
+      <c r="E11" s="23" t="str">
         <v/>
       </c>
-      <c r="F9" s="23" t="str">
+      <c r="F11" s="23" t="str">
         <v/>
       </c>
-      <c r="G9" s="24" t="str">
+      <c r="G11" s="24" t="str">
         <v/>
       </c>
-      <c r="H9" s="24">
-        <f>SUM(H4:H8)</f>
-        <v>62636</v>
-      </c>
-      <c r="I9" s="23" t="str">
+      <c r="H11" s="24">
+        <f>SUM(H4:H10)</f>
+        <v>61929</v>
+      </c>
+      <c r="I11" s="23" t="str">
         <v>1 Node(s)</v>
       </c>
-      <c r="J9" s="23" t="str">
+      <c r="J11" s="23" t="str">
         <v>CANDIDATE DOCUMENT REVIEW: PASS</v>
       </c>
-      <c r="K9" s="23" t="str">
+      <c r="K11" s="23" t="str">
         <v>LOCAL_RULE_CHECKED</v>
       </c>
-      <c r="L9" s="23" t="str">
-        <v>CLIC ACCEPTED — 2026-09-22T07:58:17.037Z</v>
+      <c r="L11" s="23" t="str">
+        <v>CLIC ACCEPTED — 2026-09-22T18:07:43.869Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>